<commit_message>
fixes de los informes
</commit_message>
<xml_diff>
--- a/public/informes-templates/INFORME DIAGNOSTICO DE EQUIPO .xlsx
+++ b/public/informes-templates/INFORME DIAGNOSTICO DE EQUIPO .xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C0C19AD-F2CB-4C82-8903-BED278494B8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88497B54-1729-437A-9CAB-80EC2CF0FF3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,39 +15,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="66">
-  <si>
-    <t>INFORME DE SERVICIO</t>
-  </si>
-  <si>
-    <t>EMPRESA / CLIENTE</t>
-  </si>
-  <si>
-    <t>CONTACTO</t>
-  </si>
-  <si>
-    <t>ORDEN DE COMPRA</t>
-  </si>
-  <si>
-    <t>COT</t>
-  </si>
-  <si>
-    <t>LINEA / AREA</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="51">
   <si>
     <t xml:space="preserve">DESCRIPCION </t>
   </si>
   <si>
-    <t>TIPO</t>
-  </si>
-  <si>
     <t>CANTIDAD</t>
-  </si>
-  <si>
-    <t>FECHA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EQUIPO 1 </t>
   </si>
   <si>
     <t>DATOS DEL EQUIPO</t>
@@ -194,32 +167,14 @@
     <t>OBSERVACION</t>
   </si>
   <si>
-    <t>1)</t>
-  </si>
-  <si>
-    <t>2)</t>
-  </si>
-  <si>
-    <t>3)</t>
-  </si>
-  <si>
     <t>RECOMENDACION</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">3) </t>
-  </si>
-  <si>
-    <t>4)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -247,22 +202,8 @@
     <font>
       <b/>
       <i/>
-      <sz val="8"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <i/>
       <sz val="9"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <i/>
-      <sz val="20"/>
-      <color theme="1"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -303,8 +244,13 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -327,6 +273,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
         <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -472,20 +424,24 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </left>
       <right style="thin">
-        <color rgb="FF000000"/>
+        <color indexed="64"/>
       </right>
-      <top/>
-      <bottom/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -493,32 +449,89 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -526,94 +539,64 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -631,55 +614,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="0" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -883,23 +817,23 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Z229"/>
+  <dimension ref="A1:Z224"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="8" width="18.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="14"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="23"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
@@ -920,14 +854,14 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15"/>
-      <c r="B2" s="16"/>
-      <c r="C2" s="16"/>
-      <c r="D2" s="16"/>
-      <c r="E2" s="16"/>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
-      <c r="H2" s="17"/>
+      <c r="A2" s="30"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="26"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
@@ -948,16 +882,14 @@
       <c r="Z2" s="1"/>
     </row>
     <row r="3" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="18"/>
-      <c r="B3" s="14"/>
-      <c r="C3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D3" s="21"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="14"/>
+      <c r="A3" s="33"/>
+      <c r="B3" s="34"/>
+      <c r="C3" s="34"/>
+      <c r="D3" s="34"/>
+      <c r="E3" s="34"/>
+      <c r="F3" s="34"/>
+      <c r="G3" s="34"/>
+      <c r="H3" s="35"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
@@ -978,16 +910,14 @@
       <c r="Z3" s="1"/>
     </row>
     <row r="4" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="19"/>
-      <c r="B4" s="20"/>
-      <c r="C4" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D4" s="21"/>
-      <c r="E4" s="13"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="13"/>
-      <c r="H4" s="14"/>
+      <c r="A4" s="28"/>
+      <c r="B4" s="25"/>
+      <c r="C4" s="25"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="25"/>
+      <c r="F4" s="25"/>
+      <c r="G4" s="25"/>
+      <c r="H4" s="25"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
@@ -1008,16 +938,16 @@
       <c r="Z4" s="1"/>
     </row>
     <row r="5" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="19"/>
-      <c r="B5" s="20"/>
-      <c r="C5" s="3" t="s">
-        <v>3</v>
+      <c r="A5" s="38" t="s">
+        <v>2</v>
       </c>
-      <c r="D5" s="21"/>
-      <c r="E5" s="13"/>
-      <c r="F5" s="13"/>
-      <c r="G5" s="13"/>
-      <c r="H5" s="14"/>
+      <c r="B5" s="46"/>
+      <c r="C5" s="46"/>
+      <c r="D5" s="46"/>
+      <c r="E5" s="46"/>
+      <c r="F5" s="46"/>
+      <c r="G5" s="46"/>
+      <c r="H5" s="39"/>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
@@ -1038,16 +968,26 @@
       <c r="Z5" s="1"/>
     </row>
     <row r="6" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="19"/>
-      <c r="B6" s="20"/>
-      <c r="C6" s="3" t="s">
+      <c r="A6" s="36" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="37"/>
+      <c r="C6" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="21"/>
-      <c r="E6" s="13"/>
-      <c r="F6" s="13"/>
-      <c r="G6" s="13"/>
-      <c r="H6" s="14"/>
+      <c r="D6" s="39"/>
+      <c r="E6" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>8</v>
+      </c>
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
@@ -1068,16 +1008,14 @@
       <c r="Z6" s="1"/>
     </row>
     <row r="7" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="19"/>
-      <c r="B7" s="20"/>
-      <c r="C7" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D7" s="21"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="13"/>
-      <c r="H7" s="14"/>
+      <c r="A7" s="40"/>
+      <c r="B7" s="41"/>
+      <c r="C7" s="42"/>
+      <c r="D7" s="43"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
@@ -1098,16 +1036,18 @@
       <c r="Z7" s="1"/>
     </row>
     <row r="8" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="19"/>
-      <c r="B8" s="20"/>
-      <c r="C8" s="3" t="s">
-        <v>6</v>
+      <c r="A8" s="10" t="s">
+        <v>9</v>
       </c>
-      <c r="D8" s="21"/>
-      <c r="E8" s="13"/>
-      <c r="F8" s="13"/>
-      <c r="G8" s="13"/>
-      <c r="H8" s="14"/>
+      <c r="B8" s="48"/>
+      <c r="C8" s="47" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" s="29"/>
+      <c r="E8" s="44"/>
+      <c r="F8" s="45"/>
+      <c r="G8" s="16"/>
+      <c r="H8" s="13"/>
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
@@ -1128,16 +1068,16 @@
       <c r="Z8" s="1"/>
     </row>
     <row r="9" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="19"/>
-      <c r="B9" s="20"/>
-      <c r="C9" s="3" t="s">
-        <v>7</v>
+      <c r="A9" s="17" t="s">
+        <v>11</v>
       </c>
-      <c r="D9" s="21"/>
-      <c r="E9" s="13"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="13"/>
-      <c r="H9" s="14"/>
+      <c r="B9" s="25"/>
+      <c r="C9" s="12"/>
+      <c r="D9" s="12"/>
+      <c r="E9" s="12"/>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="13"/>
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
@@ -1158,16 +1098,14 @@
       <c r="Z9" s="1"/>
     </row>
     <row r="10" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="19"/>
-      <c r="B10" s="20"/>
-      <c r="C10" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D10" s="21"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="13"/>
-      <c r="H10" s="14"/>
+      <c r="A10" s="49"/>
+      <c r="B10" s="50"/>
+      <c r="C10" s="49"/>
+      <c r="D10" s="50"/>
+      <c r="E10" s="49"/>
+      <c r="F10" s="50"/>
+      <c r="G10" s="49"/>
+      <c r="H10" s="50"/>
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
@@ -1188,16 +1126,14 @@
       <c r="Z10" s="1"/>
     </row>
     <row r="11" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="19"/>
-      <c r="B11" s="20"/>
-      <c r="C11" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D11" s="22"/>
-      <c r="E11" s="23"/>
-      <c r="F11" s="23"/>
-      <c r="G11" s="23"/>
-      <c r="H11" s="24"/>
+      <c r="A11" s="51"/>
+      <c r="B11" s="52"/>
+      <c r="C11" s="51"/>
+      <c r="D11" s="52"/>
+      <c r="E11" s="51"/>
+      <c r="F11" s="52"/>
+      <c r="G11" s="51"/>
+      <c r="H11" s="52"/>
       <c r="I11" s="1"/>
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
@@ -1218,14 +1154,14 @@
       <c r="Z11" s="1"/>
     </row>
     <row r="12" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="25"/>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="16"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="16"/>
-      <c r="H12" s="16"/>
+      <c r="A12" s="51"/>
+      <c r="B12" s="52"/>
+      <c r="C12" s="51"/>
+      <c r="D12" s="52"/>
+      <c r="E12" s="51"/>
+      <c r="F12" s="52"/>
+      <c r="G12" s="51"/>
+      <c r="H12" s="52"/>
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
@@ -1246,18 +1182,14 @@
       <c r="Z12" s="1"/>
     </row>
     <row r="13" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="26" t="s">
-        <v>10</v>
-      </c>
-      <c r="B13" s="14"/>
-      <c r="C13" s="27" t="s">
-        <v>11</v>
-      </c>
-      <c r="D13" s="23"/>
-      <c r="E13" s="23"/>
-      <c r="F13" s="23"/>
-      <c r="G13" s="23"/>
-      <c r="H13" s="24"/>
+      <c r="A13" s="51"/>
+      <c r="B13" s="52"/>
+      <c r="C13" s="51"/>
+      <c r="D13" s="52"/>
+      <c r="E13" s="51"/>
+      <c r="F13" s="52"/>
+      <c r="G13" s="51"/>
+      <c r="H13" s="52"/>
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
       <c r="K13" s="1"/>
@@ -1278,26 +1210,14 @@
       <c r="Z13" s="1"/>
     </row>
     <row r="14" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="19"/>
-      <c r="B14" s="20"/>
-      <c r="C14" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>17</v>
-      </c>
+      <c r="A14" s="51"/>
+      <c r="B14" s="52"/>
+      <c r="C14" s="51"/>
+      <c r="D14" s="52"/>
+      <c r="E14" s="51"/>
+      <c r="F14" s="52"/>
+      <c r="G14" s="51"/>
+      <c r="H14" s="52"/>
       <c r="I14" s="1"/>
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
@@ -1318,14 +1238,14 @@
       <c r="Z14" s="1"/>
     </row>
     <row r="15" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="19"/>
-      <c r="B15" s="20"/>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
+      <c r="A15" s="51"/>
+      <c r="B15" s="52"/>
+      <c r="C15" s="51"/>
+      <c r="D15" s="52"/>
+      <c r="E15" s="51"/>
+      <c r="F15" s="52"/>
+      <c r="G15" s="51"/>
+      <c r="H15" s="52"/>
       <c r="I15" s="1"/>
       <c r="J15" s="1"/>
       <c r="K15" s="1"/>
@@ -1346,18 +1266,14 @@
       <c r="Z15" s="1"/>
     </row>
     <row r="16" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="15"/>
-      <c r="B16" s="17"/>
-      <c r="C16" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D16" s="6"/>
-      <c r="E16" s="28" t="s">
-        <v>19</v>
-      </c>
-      <c r="F16" s="20"/>
-      <c r="G16" s="29"/>
-      <c r="H16" s="24"/>
+      <c r="A16" s="51"/>
+      <c r="B16" s="52"/>
+      <c r="C16" s="51"/>
+      <c r="D16" s="52"/>
+      <c r="E16" s="51"/>
+      <c r="F16" s="52"/>
+      <c r="G16" s="51"/>
+      <c r="H16" s="52"/>
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
       <c r="K16" s="1"/>
@@ -1378,16 +1294,14 @@
       <c r="Z16" s="1"/>
     </row>
     <row r="17" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="30" t="s">
-        <v>20</v>
-      </c>
-      <c r="B17" s="23"/>
-      <c r="C17" s="23"/>
-      <c r="D17" s="23"/>
-      <c r="E17" s="23"/>
-      <c r="F17" s="23"/>
-      <c r="G17" s="23"/>
-      <c r="H17" s="24"/>
+      <c r="A17" s="51"/>
+      <c r="B17" s="52"/>
+      <c r="C17" s="51"/>
+      <c r="D17" s="52"/>
+      <c r="E17" s="51"/>
+      <c r="F17" s="52"/>
+      <c r="G17" s="51"/>
+      <c r="H17" s="52"/>
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
       <c r="K17" s="1"/>
@@ -1408,14 +1322,14 @@
       <c r="Z17" s="1"/>
     </row>
     <row r="18" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="40"/>
-      <c r="B18" s="41"/>
-      <c r="C18" s="40"/>
-      <c r="D18" s="41"/>
-      <c r="E18" s="40"/>
-      <c r="F18" s="41"/>
-      <c r="G18" s="40"/>
-      <c r="H18" s="41"/>
+      <c r="A18" s="51"/>
+      <c r="B18" s="52"/>
+      <c r="C18" s="51"/>
+      <c r="D18" s="52"/>
+      <c r="E18" s="51"/>
+      <c r="F18" s="52"/>
+      <c r="G18" s="51"/>
+      <c r="H18" s="52"/>
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
@@ -1436,14 +1350,14 @@
       <c r="Z18" s="1"/>
     </row>
     <row r="19" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="42"/>
-      <c r="B19" s="43"/>
-      <c r="C19" s="42"/>
-      <c r="D19" s="43"/>
-      <c r="E19" s="42"/>
-      <c r="F19" s="43"/>
-      <c r="G19" s="42"/>
-      <c r="H19" s="43"/>
+      <c r="A19" s="51"/>
+      <c r="B19" s="52"/>
+      <c r="C19" s="51"/>
+      <c r="D19" s="52"/>
+      <c r="E19" s="51"/>
+      <c r="F19" s="52"/>
+      <c r="G19" s="51"/>
+      <c r="H19" s="52"/>
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
       <c r="K19" s="1"/>
@@ -1464,14 +1378,14 @@
       <c r="Z19" s="1"/>
     </row>
     <row r="20" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="42"/>
-      <c r="B20" s="43"/>
-      <c r="C20" s="42"/>
-      <c r="D20" s="43"/>
-      <c r="E20" s="42"/>
-      <c r="F20" s="43"/>
-      <c r="G20" s="42"/>
-      <c r="H20" s="43"/>
+      <c r="A20" s="51"/>
+      <c r="B20" s="52"/>
+      <c r="C20" s="51"/>
+      <c r="D20" s="52"/>
+      <c r="E20" s="51"/>
+      <c r="F20" s="52"/>
+      <c r="G20" s="51"/>
+      <c r="H20" s="52"/>
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
       <c r="K20" s="1"/>
@@ -1492,14 +1406,14 @@
       <c r="Z20" s="1"/>
     </row>
     <row r="21" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="42"/>
-      <c r="B21" s="43"/>
-      <c r="C21" s="42"/>
-      <c r="D21" s="43"/>
-      <c r="E21" s="42"/>
-      <c r="F21" s="43"/>
-      <c r="G21" s="42"/>
-      <c r="H21" s="43"/>
+      <c r="A21" s="51"/>
+      <c r="B21" s="52"/>
+      <c r="C21" s="51"/>
+      <c r="D21" s="52"/>
+      <c r="E21" s="51"/>
+      <c r="F21" s="52"/>
+      <c r="G21" s="51"/>
+      <c r="H21" s="52"/>
       <c r="I21" s="1"/>
       <c r="J21" s="1"/>
       <c r="K21" s="1"/>
@@ -1520,14 +1434,22 @@
       <c r="Z21" s="1"/>
     </row>
     <row r="22" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="42"/>
-      <c r="B22" s="43"/>
-      <c r="C22" s="42"/>
-      <c r="D22" s="43"/>
-      <c r="E22" s="42"/>
-      <c r="F22" s="43"/>
-      <c r="G22" s="42"/>
-      <c r="H22" s="43"/>
+      <c r="A22" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="B22" s="13"/>
+      <c r="C22" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="D22" s="13"/>
+      <c r="E22" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" s="13"/>
+      <c r="G22" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="H22" s="13"/>
       <c r="I22" s="1"/>
       <c r="J22" s="1"/>
       <c r="K22" s="1"/>
@@ -1548,14 +1470,14 @@
       <c r="Z22" s="1"/>
     </row>
     <row r="23" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="42"/>
-      <c r="B23" s="43"/>
-      <c r="C23" s="42"/>
-      <c r="D23" s="43"/>
-      <c r="E23" s="42"/>
-      <c r="F23" s="43"/>
-      <c r="G23" s="42"/>
-      <c r="H23" s="43"/>
+      <c r="A23" s="49"/>
+      <c r="B23" s="50"/>
+      <c r="C23" s="49"/>
+      <c r="D23" s="50"/>
+      <c r="E23" s="49"/>
+      <c r="F23" s="50"/>
+      <c r="G23" s="49"/>
+      <c r="H23" s="50"/>
       <c r="I23" s="1"/>
       <c r="J23" s="1"/>
       <c r="K23" s="1"/>
@@ -1576,14 +1498,14 @@
       <c r="Z23" s="1"/>
     </row>
     <row r="24" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="42"/>
-      <c r="B24" s="43"/>
-      <c r="C24" s="42"/>
-      <c r="D24" s="43"/>
-      <c r="E24" s="42"/>
-      <c r="F24" s="43"/>
-      <c r="G24" s="42"/>
-      <c r="H24" s="43"/>
+      <c r="A24" s="51"/>
+      <c r="B24" s="52"/>
+      <c r="C24" s="51"/>
+      <c r="D24" s="52"/>
+      <c r="E24" s="51"/>
+      <c r="F24" s="52"/>
+      <c r="G24" s="51"/>
+      <c r="H24" s="52"/>
       <c r="I24" s="1"/>
       <c r="J24" s="1"/>
       <c r="K24" s="1"/>
@@ -1604,14 +1526,14 @@
       <c r="Z24" s="1"/>
     </row>
     <row r="25" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="42"/>
-      <c r="B25" s="43"/>
-      <c r="C25" s="42"/>
-      <c r="D25" s="43"/>
-      <c r="E25" s="42"/>
-      <c r="F25" s="43"/>
-      <c r="G25" s="42"/>
-      <c r="H25" s="43"/>
+      <c r="A25" s="51"/>
+      <c r="B25" s="52"/>
+      <c r="C25" s="51"/>
+      <c r="D25" s="52"/>
+      <c r="E25" s="51"/>
+      <c r="F25" s="52"/>
+      <c r="G25" s="51"/>
+      <c r="H25" s="52"/>
       <c r="I25" s="1"/>
       <c r="J25" s="1"/>
       <c r="K25" s="1"/>
@@ -1632,14 +1554,14 @@
       <c r="Z25" s="1"/>
     </row>
     <row r="26" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="42"/>
-      <c r="B26" s="43"/>
-      <c r="C26" s="42"/>
-      <c r="D26" s="43"/>
-      <c r="E26" s="42"/>
-      <c r="F26" s="43"/>
-      <c r="G26" s="42"/>
-      <c r="H26" s="43"/>
+      <c r="A26" s="51"/>
+      <c r="B26" s="52"/>
+      <c r="C26" s="51"/>
+      <c r="D26" s="52"/>
+      <c r="E26" s="51"/>
+      <c r="F26" s="52"/>
+      <c r="G26" s="51"/>
+      <c r="H26" s="52"/>
       <c r="I26" s="1"/>
       <c r="J26" s="1"/>
       <c r="K26" s="1"/>
@@ -1660,14 +1582,14 @@
       <c r="Z26" s="1"/>
     </row>
     <row r="27" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="42"/>
-      <c r="B27" s="43"/>
-      <c r="C27" s="42"/>
-      <c r="D27" s="43"/>
-      <c r="E27" s="42"/>
-      <c r="F27" s="43"/>
-      <c r="G27" s="42"/>
-      <c r="H27" s="43"/>
+      <c r="A27" s="51"/>
+      <c r="B27" s="52"/>
+      <c r="C27" s="51"/>
+      <c r="D27" s="52"/>
+      <c r="E27" s="51"/>
+      <c r="F27" s="52"/>
+      <c r="G27" s="51"/>
+      <c r="H27" s="52"/>
       <c r="I27" s="1"/>
       <c r="J27" s="1"/>
       <c r="K27" s="1"/>
@@ -1688,14 +1610,14 @@
       <c r="Z27" s="1"/>
     </row>
     <row r="28" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="42"/>
-      <c r="B28" s="43"/>
-      <c r="C28" s="42"/>
-      <c r="D28" s="43"/>
-      <c r="E28" s="42"/>
-      <c r="F28" s="43"/>
-      <c r="G28" s="42"/>
-      <c r="H28" s="43"/>
+      <c r="A28" s="51"/>
+      <c r="B28" s="52"/>
+      <c r="C28" s="51"/>
+      <c r="D28" s="52"/>
+      <c r="E28" s="51"/>
+      <c r="F28" s="52"/>
+      <c r="G28" s="51"/>
+      <c r="H28" s="52"/>
       <c r="I28" s="1"/>
       <c r="J28" s="1"/>
       <c r="K28" s="1"/>
@@ -1716,14 +1638,14 @@
       <c r="Z28" s="1"/>
     </row>
     <row r="29" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="42"/>
-      <c r="B29" s="43"/>
-      <c r="C29" s="42"/>
-      <c r="D29" s="43"/>
-      <c r="E29" s="42"/>
-      <c r="F29" s="43"/>
-      <c r="G29" s="42"/>
-      <c r="H29" s="43"/>
+      <c r="A29" s="51"/>
+      <c r="B29" s="52"/>
+      <c r="C29" s="51"/>
+      <c r="D29" s="52"/>
+      <c r="E29" s="51"/>
+      <c r="F29" s="52"/>
+      <c r="G29" s="51"/>
+      <c r="H29" s="52"/>
       <c r="I29" s="1"/>
       <c r="J29" s="1"/>
       <c r="K29" s="1"/>
@@ -1744,22 +1666,14 @@
       <c r="Z29" s="1"/>
     </row>
     <row r="30" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="31" t="s">
-        <v>21</v>
-      </c>
-      <c r="B30" s="24"/>
-      <c r="C30" s="31" t="s">
-        <v>22</v>
-      </c>
-      <c r="D30" s="24"/>
-      <c r="E30" s="31" t="s">
-        <v>23</v>
-      </c>
-      <c r="F30" s="24"/>
-      <c r="G30" s="31" t="s">
-        <v>23</v>
-      </c>
-      <c r="H30" s="24"/>
+      <c r="A30" s="51"/>
+      <c r="B30" s="52"/>
+      <c r="C30" s="51"/>
+      <c r="D30" s="52"/>
+      <c r="E30" s="51"/>
+      <c r="F30" s="52"/>
+      <c r="G30" s="51"/>
+      <c r="H30" s="52"/>
       <c r="I30" s="1"/>
       <c r="J30" s="1"/>
       <c r="K30" s="1"/>
@@ -1779,15 +1693,15 @@
       <c r="Y30" s="1"/>
       <c r="Z30" s="1"/>
     </row>
-    <row r="31" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="40"/>
-      <c r="B31" s="41"/>
-      <c r="C31" s="40"/>
-      <c r="D31" s="41"/>
-      <c r="E31" s="40"/>
-      <c r="F31" s="41"/>
-      <c r="G31" s="40"/>
-      <c r="H31" s="41"/>
+    <row r="31" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="51"/>
+      <c r="B31" s="52"/>
+      <c r="C31" s="51"/>
+      <c r="D31" s="52"/>
+      <c r="E31" s="51"/>
+      <c r="F31" s="52"/>
+      <c r="G31" s="51"/>
+      <c r="H31" s="52"/>
       <c r="I31" s="1"/>
       <c r="J31" s="1"/>
       <c r="K31" s="1"/>
@@ -1807,15 +1721,15 @@
       <c r="Y31" s="1"/>
       <c r="Z31" s="1"/>
     </row>
-    <row r="32" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="42"/>
-      <c r="B32" s="43"/>
-      <c r="C32" s="42"/>
-      <c r="D32" s="43"/>
-      <c r="E32" s="42"/>
-      <c r="F32" s="43"/>
-      <c r="G32" s="42"/>
-      <c r="H32" s="43"/>
+    <row r="32" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="51"/>
+      <c r="B32" s="52"/>
+      <c r="C32" s="51"/>
+      <c r="D32" s="52"/>
+      <c r="E32" s="51"/>
+      <c r="F32" s="52"/>
+      <c r="G32" s="51"/>
+      <c r="H32" s="52"/>
       <c r="I32" s="1"/>
       <c r="J32" s="1"/>
       <c r="K32" s="1"/>
@@ -1835,15 +1749,15 @@
       <c r="Y32" s="1"/>
       <c r="Z32" s="1"/>
     </row>
-    <row r="33" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="42"/>
-      <c r="B33" s="43"/>
-      <c r="C33" s="42"/>
-      <c r="D33" s="43"/>
-      <c r="E33" s="42"/>
-      <c r="F33" s="43"/>
-      <c r="G33" s="42"/>
-      <c r="H33" s="43"/>
+    <row r="33" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="51"/>
+      <c r="B33" s="52"/>
+      <c r="C33" s="51"/>
+      <c r="D33" s="52"/>
+      <c r="E33" s="51"/>
+      <c r="F33" s="52"/>
+      <c r="G33" s="51"/>
+      <c r="H33" s="52"/>
       <c r="I33" s="1"/>
       <c r="J33" s="1"/>
       <c r="K33" s="1"/>
@@ -1863,15 +1777,15 @@
       <c r="Y33" s="1"/>
       <c r="Z33" s="1"/>
     </row>
-    <row r="34" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="42"/>
-      <c r="B34" s="43"/>
-      <c r="C34" s="42"/>
-      <c r="D34" s="43"/>
-      <c r="E34" s="42"/>
-      <c r="F34" s="43"/>
-      <c r="G34" s="42"/>
-      <c r="H34" s="43"/>
+    <row r="34" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="51"/>
+      <c r="B34" s="52"/>
+      <c r="C34" s="51"/>
+      <c r="D34" s="52"/>
+      <c r="E34" s="51"/>
+      <c r="F34" s="52"/>
+      <c r="G34" s="51"/>
+      <c r="H34" s="52"/>
       <c r="I34" s="1"/>
       <c r="J34" s="1"/>
       <c r="K34" s="1"/>
@@ -1891,15 +1805,23 @@
       <c r="Y34" s="1"/>
       <c r="Z34" s="1"/>
     </row>
-    <row r="35" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="42"/>
-      <c r="B35" s="43"/>
-      <c r="C35" s="42"/>
-      <c r="D35" s="43"/>
-      <c r="E35" s="42"/>
-      <c r="F35" s="43"/>
-      <c r="G35" s="42"/>
-      <c r="H35" s="43"/>
+    <row r="35" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="B35" s="23"/>
+      <c r="C35" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="D35" s="23"/>
+      <c r="E35" s="22" t="s">
+        <v>17</v>
+      </c>
+      <c r="F35" s="23"/>
+      <c r="G35" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="H35" s="13"/>
       <c r="I35" s="1"/>
       <c r="J35" s="1"/>
       <c r="K35" s="1"/>
@@ -1919,15 +1841,15 @@
       <c r="Y35" s="1"/>
       <c r="Z35" s="1"/>
     </row>
-    <row r="36" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="42"/>
-      <c r="B36" s="43"/>
-      <c r="C36" s="42"/>
-      <c r="D36" s="43"/>
-      <c r="E36" s="42"/>
-      <c r="F36" s="43"/>
-      <c r="G36" s="42"/>
-      <c r="H36" s="43"/>
+    <row r="36" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="1"/>
+      <c r="B36" s="1"/>
+      <c r="C36" s="1"/>
+      <c r="D36" s="1"/>
+      <c r="E36" s="1"/>
+      <c r="F36" s="1"/>
+      <c r="G36" s="1"/>
+      <c r="H36" s="1"/>
       <c r="I36" s="1"/>
       <c r="J36" s="1"/>
       <c r="K36" s="1"/>
@@ -1947,15 +1869,18 @@
       <c r="Y36" s="1"/>
       <c r="Z36" s="1"/>
     </row>
-    <row r="37" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="42"/>
-      <c r="B37" s="43"/>
-      <c r="C37" s="42"/>
-      <c r="D37" s="43"/>
-      <c r="E37" s="42"/>
-      <c r="F37" s="43"/>
-      <c r="G37" s="42"/>
-      <c r="H37" s="43"/>
+    <row r="37" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="B37" s="25"/>
+      <c r="C37" s="26"/>
+      <c r="E37" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="F37" s="12"/>
+      <c r="G37" s="12"/>
+      <c r="H37" s="13"/>
       <c r="I37" s="1"/>
       <c r="J37" s="1"/>
       <c r="K37" s="1"/>
@@ -1975,18 +1900,24 @@
       <c r="Y37" s="1"/>
       <c r="Z37" s="1"/>
     </row>
-    <row r="38" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="42"/>
-      <c r="B38" s="43"/>
-      <c r="C38" s="42"/>
-      <c r="D38" s="43"/>
-      <c r="E38" s="42"/>
-      <c r="F38" s="43"/>
-      <c r="G38" s="42"/>
-      <c r="H38" s="43"/>
-      <c r="I38" s="1"/>
-      <c r="J38" s="1"/>
-      <c r="K38" s="1"/>
+    <row r="38" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E38" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="F38" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="G38" s="12"/>
+      <c r="H38" s="13"/>
       <c r="L38" s="1"/>
       <c r="M38" s="1"/>
       <c r="N38" s="1"/>
@@ -2004,17 +1935,15 @@
       <c r="Z38" s="1"/>
     </row>
     <row r="39" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="42"/>
-      <c r="B39" s="43"/>
-      <c r="C39" s="42"/>
-      <c r="D39" s="43"/>
-      <c r="E39" s="42"/>
-      <c r="F39" s="43"/>
-      <c r="G39" s="42"/>
-      <c r="H39" s="43"/>
-      <c r="I39" s="1"/>
-      <c r="J39" s="1"/>
-      <c r="K39" s="1"/>
+      <c r="A39" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B39" s="7"/>
+      <c r="C39" s="7"/>
+      <c r="E39" s="8"/>
+      <c r="F39" s="19"/>
+      <c r="G39" s="12"/>
+      <c r="H39" s="13"/>
       <c r="L39" s="1"/>
       <c r="M39" s="1"/>
       <c r="N39" s="1"/>
@@ -2032,17 +1961,15 @@
       <c r="Z39" s="1"/>
     </row>
     <row r="40" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="42"/>
-      <c r="B40" s="43"/>
-      <c r="C40" s="42"/>
-      <c r="D40" s="43"/>
-      <c r="E40" s="42"/>
-      <c r="F40" s="43"/>
-      <c r="G40" s="42"/>
-      <c r="H40" s="43"/>
-      <c r="I40" s="1"/>
-      <c r="J40" s="1"/>
-      <c r="K40" s="1"/>
+      <c r="A40" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B40" s="7"/>
+      <c r="C40" s="7"/>
+      <c r="E40" s="8"/>
+      <c r="F40" s="19"/>
+      <c r="G40" s="12"/>
+      <c r="H40" s="13"/>
       <c r="L40" s="1"/>
       <c r="M40" s="1"/>
       <c r="N40" s="1"/>
@@ -2060,17 +1987,15 @@
       <c r="Z40" s="1"/>
     </row>
     <row r="41" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="42"/>
-      <c r="B41" s="43"/>
-      <c r="C41" s="42"/>
-      <c r="D41" s="43"/>
-      <c r="E41" s="42"/>
-      <c r="F41" s="43"/>
-      <c r="G41" s="42"/>
-      <c r="H41" s="43"/>
-      <c r="I41" s="1"/>
-      <c r="J41" s="1"/>
-      <c r="K41" s="1"/>
+      <c r="A41" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B41" s="7"/>
+      <c r="C41" s="7"/>
+      <c r="E41" s="8"/>
+      <c r="F41" s="19"/>
+      <c r="G41" s="12"/>
+      <c r="H41" s="13"/>
       <c r="L41" s="1"/>
       <c r="M41" s="1"/>
       <c r="N41" s="1"/>
@@ -2088,17 +2013,15 @@
       <c r="Z41" s="1"/>
     </row>
     <row r="42" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="42"/>
-      <c r="B42" s="43"/>
-      <c r="C42" s="42"/>
-      <c r="D42" s="43"/>
-      <c r="E42" s="42"/>
-      <c r="F42" s="43"/>
-      <c r="G42" s="42"/>
-      <c r="H42" s="43"/>
-      <c r="I42" s="1"/>
-      <c r="J42" s="1"/>
-      <c r="K42" s="1"/>
+      <c r="A42" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B42" s="7"/>
+      <c r="C42" s="7"/>
+      <c r="E42" s="8"/>
+      <c r="F42" s="19"/>
+      <c r="G42" s="12"/>
+      <c r="H42" s="13"/>
       <c r="L42" s="1"/>
       <c r="M42" s="1"/>
       <c r="N42" s="1"/>
@@ -2116,25 +2039,15 @@
       <c r="Z42" s="1"/>
     </row>
     <row r="43" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="32" t="s">
-        <v>24</v>
+      <c r="A43" s="6" t="s">
+        <v>29</v>
       </c>
-      <c r="B43" s="14"/>
-      <c r="C43" s="32" t="s">
-        <v>25</v>
-      </c>
-      <c r="D43" s="14"/>
-      <c r="E43" s="32" t="s">
-        <v>26</v>
-      </c>
-      <c r="F43" s="14"/>
-      <c r="G43" s="31" t="s">
-        <v>27</v>
-      </c>
-      <c r="H43" s="24"/>
-      <c r="I43" s="1"/>
-      <c r="J43" s="1"/>
-      <c r="K43" s="1"/>
+      <c r="B43" s="7"/>
+      <c r="C43" s="7"/>
+      <c r="E43" s="8"/>
+      <c r="F43" s="19"/>
+      <c r="G43" s="12"/>
+      <c r="H43" s="13"/>
       <c r="L43" s="1"/>
       <c r="M43" s="1"/>
       <c r="N43" s="1"/>
@@ -2152,17 +2065,15 @@
       <c r="Z43" s="1"/>
     </row>
     <row r="44" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="1"/>
-      <c r="B44" s="1"/>
-      <c r="C44" s="1"/>
-      <c r="D44" s="1"/>
-      <c r="E44" s="1"/>
-      <c r="F44" s="1"/>
-      <c r="G44" s="1"/>
-      <c r="H44" s="1"/>
-      <c r="I44" s="1"/>
-      <c r="J44" s="1"/>
-      <c r="K44" s="1"/>
+      <c r="A44" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B44" s="7"/>
+      <c r="C44" s="7"/>
+      <c r="E44" s="8"/>
+      <c r="F44" s="19"/>
+      <c r="G44" s="12"/>
+      <c r="H44" s="13"/>
       <c r="L44" s="1"/>
       <c r="M44" s="1"/>
       <c r="N44" s="1"/>
@@ -2180,20 +2091,15 @@
       <c r="Z44" s="1"/>
     </row>
     <row r="45" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="33" t="s">
-        <v>28</v>
+      <c r="A45" s="6" t="s">
+        <v>31</v>
       </c>
-      <c r="B45" s="16"/>
-      <c r="C45" s="17"/>
-      <c r="E45" s="34" t="s">
-        <v>29</v>
-      </c>
-      <c r="F45" s="23"/>
-      <c r="G45" s="23"/>
-      <c r="H45" s="24"/>
-      <c r="I45" s="1"/>
-      <c r="J45" s="1"/>
-      <c r="K45" s="1"/>
+      <c r="B45" s="7"/>
+      <c r="C45" s="7"/>
+      <c r="E45" s="8"/>
+      <c r="F45" s="19"/>
+      <c r="G45" s="12"/>
+      <c r="H45" s="13"/>
       <c r="L45" s="1"/>
       <c r="M45" s="1"/>
       <c r="N45" s="1"/>
@@ -2211,23 +2117,15 @@
       <c r="Z45" s="1"/>
     </row>
     <row r="46" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="B46" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="C46" s="7" t="s">
+      <c r="A46" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="E46" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="F46" s="31" t="s">
-        <v>33</v>
-      </c>
-      <c r="G46" s="23"/>
-      <c r="H46" s="24"/>
+      <c r="B46" s="20"/>
+      <c r="C46" s="13"/>
+      <c r="E46" s="8"/>
+      <c r="F46" s="19"/>
+      <c r="G46" s="12"/>
+      <c r="H46" s="13"/>
       <c r="L46" s="1"/>
       <c r="M46" s="1"/>
       <c r="N46" s="1"/>
@@ -2245,15 +2143,14 @@
       <c r="Z46" s="1"/>
     </row>
     <row r="47" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="B47" s="9"/>
-      <c r="C47" s="9"/>
-      <c r="E47" s="10"/>
-      <c r="F47" s="35"/>
-      <c r="G47" s="23"/>
-      <c r="H47" s="24"/>
+      <c r="A47" s="1"/>
+      <c r="B47" s="1"/>
+      <c r="C47" s="1"/>
+      <c r="D47" s="1"/>
+      <c r="E47" s="1"/>
+      <c r="F47" s="1"/>
+      <c r="G47" s="1"/>
+      <c r="H47" s="1"/>
       <c r="L47" s="1"/>
       <c r="M47" s="1"/>
       <c r="N47" s="1"/>
@@ -2271,15 +2168,16 @@
       <c r="Z47" s="1"/>
     </row>
     <row r="48" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="8" t="s">
-        <v>35</v>
+      <c r="A48" s="17" t="s">
+        <v>33</v>
       </c>
-      <c r="B48" s="9"/>
-      <c r="C48" s="9"/>
-      <c r="E48" s="10"/>
-      <c r="F48" s="35"/>
-      <c r="G48" s="23"/>
-      <c r="H48" s="24"/>
+      <c r="B48" s="12"/>
+      <c r="C48" s="12"/>
+      <c r="D48" s="12"/>
+      <c r="E48" s="12"/>
+      <c r="F48" s="12"/>
+      <c r="G48" s="12"/>
+      <c r="H48" s="13"/>
       <c r="L48" s="1"/>
       <c r="M48" s="1"/>
       <c r="N48" s="1"/>
@@ -2297,15 +2195,20 @@
       <c r="Z48" s="1"/>
     </row>
     <row r="49" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="8" t="s">
+      <c r="A49" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B49" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="C49" s="12"/>
+      <c r="D49" s="12"/>
+      <c r="E49" s="12"/>
+      <c r="F49" s="12"/>
+      <c r="G49" s="13"/>
+      <c r="H49" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B49" s="9"/>
-      <c r="C49" s="9"/>
-      <c r="E49" s="10"/>
-      <c r="F49" s="35"/>
-      <c r="G49" s="23"/>
-      <c r="H49" s="24"/>
       <c r="L49" s="1"/>
       <c r="M49" s="1"/>
       <c r="N49" s="1"/>
@@ -2323,15 +2226,21 @@
       <c r="Z49" s="1"/>
     </row>
     <row r="50" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="8" t="s">
+      <c r="A50" s="9">
+        <v>1</v>
+      </c>
+      <c r="B50" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="B50" s="9"/>
-      <c r="C50" s="9"/>
-      <c r="E50" s="10"/>
-      <c r="F50" s="35"/>
-      <c r="G50" s="23"/>
-      <c r="H50" s="24"/>
+      <c r="C50" s="12"/>
+      <c r="D50" s="12"/>
+      <c r="E50" s="12"/>
+      <c r="F50" s="12"/>
+      <c r="G50" s="13"/>
+      <c r="H50" s="9"/>
+      <c r="I50" s="1"/>
+      <c r="J50" s="1"/>
+      <c r="K50" s="1"/>
       <c r="L50" s="1"/>
       <c r="M50" s="1"/>
       <c r="N50" s="1"/>
@@ -2349,15 +2258,21 @@
       <c r="Z50" s="1"/>
     </row>
     <row r="51" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="8" t="s">
+      <c r="A51" s="9">
+        <v>2</v>
+      </c>
+      <c r="B51" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="B51" s="9"/>
-      <c r="C51" s="9"/>
-      <c r="E51" s="10"/>
-      <c r="F51" s="35"/>
-      <c r="G51" s="23"/>
-      <c r="H51" s="24"/>
+      <c r="C51" s="12"/>
+      <c r="D51" s="12"/>
+      <c r="E51" s="12"/>
+      <c r="F51" s="12"/>
+      <c r="G51" s="13"/>
+      <c r="H51" s="9"/>
+      <c r="I51" s="1"/>
+      <c r="J51" s="1"/>
+      <c r="K51" s="1"/>
       <c r="L51" s="1"/>
       <c r="M51" s="1"/>
       <c r="N51" s="1"/>
@@ -2375,15 +2290,21 @@
       <c r="Z51" s="1"/>
     </row>
     <row r="52" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="8" t="s">
+      <c r="A52" s="9">
+        <v>3</v>
+      </c>
+      <c r="B52" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="B52" s="9"/>
-      <c r="C52" s="9"/>
-      <c r="E52" s="10"/>
-      <c r="F52" s="35"/>
-      <c r="G52" s="23"/>
-      <c r="H52" s="24"/>
+      <c r="C52" s="12"/>
+      <c r="D52" s="12"/>
+      <c r="E52" s="12"/>
+      <c r="F52" s="12"/>
+      <c r="G52" s="13"/>
+      <c r="H52" s="9"/>
+      <c r="I52" s="1"/>
+      <c r="J52" s="1"/>
+      <c r="K52" s="1"/>
       <c r="L52" s="1"/>
       <c r="M52" s="1"/>
       <c r="N52" s="1"/>
@@ -2401,15 +2322,21 @@
       <c r="Z52" s="1"/>
     </row>
     <row r="53" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="8" t="s">
+      <c r="A53" s="9">
+        <v>4</v>
+      </c>
+      <c r="B53" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="B53" s="9"/>
-      <c r="C53" s="9"/>
-      <c r="E53" s="10"/>
-      <c r="F53" s="35"/>
-      <c r="G53" s="23"/>
-      <c r="H53" s="24"/>
+      <c r="C53" s="12"/>
+      <c r="D53" s="12"/>
+      <c r="E53" s="12"/>
+      <c r="F53" s="12"/>
+      <c r="G53" s="13"/>
+      <c r="H53" s="9"/>
+      <c r="I53" s="1"/>
+      <c r="J53" s="1"/>
+      <c r="K53" s="1"/>
       <c r="L53" s="1"/>
       <c r="M53" s="1"/>
       <c r="N53" s="1"/>
@@ -2427,15 +2354,21 @@
       <c r="Z53" s="1"/>
     </row>
     <row r="54" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="7" t="s">
+      <c r="A54" s="9">
+        <v>5</v>
+      </c>
+      <c r="B54" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="B54" s="36"/>
-      <c r="C54" s="24"/>
-      <c r="E54" s="10"/>
-      <c r="F54" s="35"/>
-      <c r="G54" s="23"/>
-      <c r="H54" s="24"/>
+      <c r="C54" s="12"/>
+      <c r="D54" s="12"/>
+      <c r="E54" s="12"/>
+      <c r="F54" s="12"/>
+      <c r="G54" s="13"/>
+      <c r="H54" s="9"/>
+      <c r="I54" s="1"/>
+      <c r="J54" s="1"/>
+      <c r="K54" s="1"/>
       <c r="L54" s="1"/>
       <c r="M54" s="1"/>
       <c r="N54" s="1"/>
@@ -2453,14 +2386,21 @@
       <c r="Z54" s="1"/>
     </row>
     <row r="55" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="1"/>
-      <c r="B55" s="1"/>
-      <c r="C55" s="1"/>
-      <c r="D55" s="1"/>
-      <c r="E55" s="1"/>
-      <c r="F55" s="1"/>
-      <c r="G55" s="1"/>
-      <c r="H55" s="1"/>
+      <c r="A55" s="9">
+        <v>6</v>
+      </c>
+      <c r="B55" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="C55" s="12"/>
+      <c r="D55" s="12"/>
+      <c r="E55" s="12"/>
+      <c r="F55" s="12"/>
+      <c r="G55" s="13"/>
+      <c r="H55" s="9"/>
+      <c r="I55" s="1"/>
+      <c r="J55" s="1"/>
+      <c r="K55" s="1"/>
       <c r="L55" s="1"/>
       <c r="M55" s="1"/>
       <c r="N55" s="1"/>
@@ -2478,16 +2418,21 @@
       <c r="Z55" s="1"/>
     </row>
     <row r="56" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="30" t="s">
-        <v>42</v>
+      <c r="A56" s="9">
+        <v>7</v>
       </c>
-      <c r="B56" s="23"/>
-      <c r="C56" s="23"/>
-      <c r="D56" s="23"/>
-      <c r="E56" s="23"/>
-      <c r="F56" s="23"/>
-      <c r="G56" s="23"/>
-      <c r="H56" s="24"/>
+      <c r="B56" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="C56" s="12"/>
+      <c r="D56" s="12"/>
+      <c r="E56" s="12"/>
+      <c r="F56" s="12"/>
+      <c r="G56" s="13"/>
+      <c r="H56" s="9"/>
+      <c r="I56" s="1"/>
+      <c r="J56" s="1"/>
+      <c r="K56" s="1"/>
       <c r="L56" s="1"/>
       <c r="M56" s="1"/>
       <c r="N56" s="1"/>
@@ -2505,20 +2450,21 @@
       <c r="Z56" s="1"/>
     </row>
     <row r="57" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="3" t="s">
-        <v>43</v>
+      <c r="A57" s="9">
+        <v>8</v>
       </c>
-      <c r="B57" s="27" t="s">
+      <c r="B57" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="C57" s="23"/>
-      <c r="D57" s="23"/>
-      <c r="E57" s="23"/>
-      <c r="F57" s="23"/>
-      <c r="G57" s="24"/>
-      <c r="H57" s="3" t="s">
-        <v>45</v>
-      </c>
+      <c r="C57" s="12"/>
+      <c r="D57" s="12"/>
+      <c r="E57" s="12"/>
+      <c r="F57" s="12"/>
+      <c r="G57" s="13"/>
+      <c r="H57" s="9"/>
+      <c r="I57" s="1"/>
+      <c r="J57" s="1"/>
+      <c r="K57" s="1"/>
       <c r="L57" s="1"/>
       <c r="M57" s="1"/>
       <c r="N57" s="1"/>
@@ -2536,18 +2482,18 @@
       <c r="Z57" s="1"/>
     </row>
     <row r="58" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="11">
-        <v>1</v>
+      <c r="A58" s="9">
+        <v>9</v>
       </c>
-      <c r="B58" s="29" t="s">
-        <v>46</v>
+      <c r="B58" s="16" t="s">
+        <v>45</v>
       </c>
-      <c r="C58" s="23"/>
-      <c r="D58" s="23"/>
-      <c r="E58" s="23"/>
-      <c r="F58" s="23"/>
-      <c r="G58" s="24"/>
-      <c r="H58" s="11"/>
+      <c r="C58" s="12"/>
+      <c r="D58" s="12"/>
+      <c r="E58" s="12"/>
+      <c r="F58" s="12"/>
+      <c r="G58" s="13"/>
+      <c r="H58" s="9"/>
       <c r="I58" s="1"/>
       <c r="J58" s="1"/>
       <c r="K58" s="1"/>
@@ -2568,18 +2514,18 @@
       <c r="Z58" s="1"/>
     </row>
     <row r="59" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="11">
-        <v>2</v>
+      <c r="A59" s="9">
+        <v>10</v>
       </c>
-      <c r="B59" s="29" t="s">
-        <v>47</v>
+      <c r="B59" s="16" t="s">
+        <v>46</v>
       </c>
-      <c r="C59" s="23"/>
-      <c r="D59" s="23"/>
-      <c r="E59" s="23"/>
-      <c r="F59" s="23"/>
-      <c r="G59" s="24"/>
-      <c r="H59" s="11"/>
+      <c r="C59" s="12"/>
+      <c r="D59" s="12"/>
+      <c r="E59" s="12"/>
+      <c r="F59" s="12"/>
+      <c r="G59" s="13"/>
+      <c r="H59" s="9"/>
       <c r="I59" s="1"/>
       <c r="J59" s="1"/>
       <c r="K59" s="1"/>
@@ -2600,18 +2546,18 @@
       <c r="Z59" s="1"/>
     </row>
     <row r="60" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="11">
-        <v>3</v>
+      <c r="A60" s="9">
+        <v>11</v>
       </c>
-      <c r="B60" s="29" t="s">
-        <v>48</v>
+      <c r="B60" s="16" t="s">
+        <v>47</v>
       </c>
-      <c r="C60" s="23"/>
-      <c r="D60" s="23"/>
-      <c r="E60" s="23"/>
-      <c r="F60" s="23"/>
-      <c r="G60" s="24"/>
-      <c r="H60" s="11"/>
+      <c r="C60" s="12"/>
+      <c r="D60" s="12"/>
+      <c r="E60" s="12"/>
+      <c r="F60" s="12"/>
+      <c r="G60" s="13"/>
+      <c r="H60" s="9"/>
       <c r="I60" s="1"/>
       <c r="J60" s="1"/>
       <c r="K60" s="1"/>
@@ -2632,18 +2578,18 @@
       <c r="Z60" s="1"/>
     </row>
     <row r="61" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="11">
-        <v>4</v>
+      <c r="A61" s="9">
+        <v>12</v>
       </c>
-      <c r="B61" s="29" t="s">
-        <v>49</v>
+      <c r="B61" s="16" t="s">
+        <v>48</v>
       </c>
-      <c r="C61" s="23"/>
-      <c r="D61" s="23"/>
-      <c r="E61" s="23"/>
-      <c r="F61" s="23"/>
-      <c r="G61" s="24"/>
-      <c r="H61" s="11"/>
+      <c r="C61" s="12"/>
+      <c r="D61" s="12"/>
+      <c r="E61" s="12"/>
+      <c r="F61" s="12"/>
+      <c r="G61" s="13"/>
+      <c r="H61" s="9"/>
       <c r="I61" s="1"/>
       <c r="J61" s="1"/>
       <c r="K61" s="1"/>
@@ -2664,18 +2610,16 @@
       <c r="Z61" s="1"/>
     </row>
     <row r="62" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="11">
-        <v>5</v>
+      <c r="A62" s="15" t="s">
+        <v>49</v>
       </c>
-      <c r="B62" s="29" t="s">
-        <v>50</v>
-      </c>
-      <c r="C62" s="23"/>
-      <c r="D62" s="23"/>
-      <c r="E62" s="23"/>
-      <c r="F62" s="23"/>
-      <c r="G62" s="24"/>
-      <c r="H62" s="11"/>
+      <c r="B62" s="12"/>
+      <c r="C62" s="12"/>
+      <c r="D62" s="12"/>
+      <c r="E62" s="12"/>
+      <c r="F62" s="12"/>
+      <c r="G62" s="12"/>
+      <c r="H62" s="13"/>
       <c r="I62" s="1"/>
       <c r="J62" s="1"/>
       <c r="K62" s="1"/>
@@ -2696,18 +2640,14 @@
       <c r="Z62" s="1"/>
     </row>
     <row r="63" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="11">
-        <v>6</v>
-      </c>
-      <c r="B63" s="29" t="s">
-        <v>51</v>
-      </c>
-      <c r="C63" s="23"/>
-      <c r="D63" s="23"/>
-      <c r="E63" s="23"/>
-      <c r="F63" s="23"/>
-      <c r="G63" s="24"/>
-      <c r="H63" s="11"/>
+      <c r="A63" s="11"/>
+      <c r="B63" s="12"/>
+      <c r="C63" s="12"/>
+      <c r="D63" s="12"/>
+      <c r="E63" s="12"/>
+      <c r="F63" s="12"/>
+      <c r="G63" s="12"/>
+      <c r="H63" s="13"/>
       <c r="I63" s="1"/>
       <c r="J63" s="1"/>
       <c r="K63" s="1"/>
@@ -2728,18 +2668,14 @@
       <c r="Z63" s="1"/>
     </row>
     <row r="64" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="11">
-        <v>7</v>
-      </c>
-      <c r="B64" s="29" t="s">
-        <v>52</v>
-      </c>
-      <c r="C64" s="23"/>
-      <c r="D64" s="23"/>
-      <c r="E64" s="23"/>
-      <c r="F64" s="23"/>
-      <c r="G64" s="24"/>
-      <c r="H64" s="11"/>
+      <c r="A64" s="11"/>
+      <c r="B64" s="12"/>
+      <c r="C64" s="12"/>
+      <c r="D64" s="12"/>
+      <c r="E64" s="12"/>
+      <c r="F64" s="12"/>
+      <c r="G64" s="12"/>
+      <c r="H64" s="13"/>
       <c r="I64" s="1"/>
       <c r="J64" s="1"/>
       <c r="K64" s="1"/>
@@ -2760,18 +2696,14 @@
       <c r="Z64" s="1"/>
     </row>
     <row r="65" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="11">
-        <v>8</v>
-      </c>
-      <c r="B65" s="29" t="s">
-        <v>53</v>
-      </c>
-      <c r="C65" s="23"/>
-      <c r="D65" s="23"/>
-      <c r="E65" s="23"/>
-      <c r="F65" s="23"/>
-      <c r="G65" s="24"/>
-      <c r="H65" s="11"/>
+      <c r="A65" s="11"/>
+      <c r="B65" s="12"/>
+      <c r="C65" s="12"/>
+      <c r="D65" s="12"/>
+      <c r="E65" s="12"/>
+      <c r="F65" s="12"/>
+      <c r="G65" s="12"/>
+      <c r="H65" s="13"/>
       <c r="I65" s="1"/>
       <c r="J65" s="1"/>
       <c r="K65" s="1"/>
@@ -2792,18 +2724,14 @@
       <c r="Z65" s="1"/>
     </row>
     <row r="66" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="11">
-        <v>9</v>
-      </c>
-      <c r="B66" s="29" t="s">
-        <v>54</v>
-      </c>
-      <c r="C66" s="23"/>
-      <c r="D66" s="23"/>
-      <c r="E66" s="23"/>
-      <c r="F66" s="23"/>
-      <c r="G66" s="24"/>
-      <c r="H66" s="11"/>
+      <c r="A66" s="11"/>
+      <c r="B66" s="12"/>
+      <c r="C66" s="12"/>
+      <c r="D66" s="12"/>
+      <c r="E66" s="12"/>
+      <c r="F66" s="12"/>
+      <c r="G66" s="12"/>
+      <c r="H66" s="13"/>
       <c r="I66" s="1"/>
       <c r="J66" s="1"/>
       <c r="K66" s="1"/>
@@ -2824,18 +2752,14 @@
       <c r="Z66" s="1"/>
     </row>
     <row r="67" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="11">
-        <v>10</v>
-      </c>
-      <c r="B67" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="C67" s="23"/>
-      <c r="D67" s="23"/>
-      <c r="E67" s="23"/>
-      <c r="F67" s="23"/>
-      <c r="G67" s="24"/>
-      <c r="H67" s="11"/>
+      <c r="A67" s="11"/>
+      <c r="B67" s="12"/>
+      <c r="C67" s="12"/>
+      <c r="D67" s="12"/>
+      <c r="E67" s="12"/>
+      <c r="F67" s="12"/>
+      <c r="G67" s="12"/>
+      <c r="H67" s="13"/>
       <c r="I67" s="1"/>
       <c r="J67" s="1"/>
       <c r="K67" s="1"/>
@@ -2856,18 +2780,16 @@
       <c r="Z67" s="1"/>
     </row>
     <row r="68" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="11">
-        <v>11</v>
+      <c r="A68" s="15" t="s">
+        <v>50</v>
       </c>
-      <c r="B68" s="29" t="s">
-        <v>56</v>
-      </c>
-      <c r="C68" s="23"/>
-      <c r="D68" s="23"/>
-      <c r="E68" s="23"/>
-      <c r="F68" s="23"/>
-      <c r="G68" s="24"/>
-      <c r="H68" s="11"/>
+      <c r="B68" s="12"/>
+      <c r="C68" s="12"/>
+      <c r="D68" s="12"/>
+      <c r="E68" s="12"/>
+      <c r="F68" s="12"/>
+      <c r="G68" s="12"/>
+      <c r="H68" s="13"/>
       <c r="I68" s="1"/>
       <c r="J68" s="1"/>
       <c r="K68" s="1"/>
@@ -2888,18 +2810,14 @@
       <c r="Z68" s="1"/>
     </row>
     <row r="69" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="11">
-        <v>12</v>
-      </c>
-      <c r="B69" s="29" t="s">
-        <v>57</v>
-      </c>
-      <c r="C69" s="23"/>
-      <c r="D69" s="23"/>
-      <c r="E69" s="23"/>
-      <c r="F69" s="23"/>
-      <c r="G69" s="24"/>
-      <c r="H69" s="11"/>
+      <c r="A69" s="11"/>
+      <c r="B69" s="12"/>
+      <c r="C69" s="12"/>
+      <c r="D69" s="12"/>
+      <c r="E69" s="12"/>
+      <c r="F69" s="12"/>
+      <c r="G69" s="12"/>
+      <c r="H69" s="13"/>
       <c r="I69" s="1"/>
       <c r="J69" s="1"/>
       <c r="K69" s="1"/>
@@ -2920,16 +2838,14 @@
       <c r="Z69" s="1"/>
     </row>
     <row r="70" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="37" t="s">
-        <v>58</v>
-      </c>
-      <c r="B70" s="23"/>
-      <c r="C70" s="23"/>
-      <c r="D70" s="23"/>
-      <c r="E70" s="23"/>
-      <c r="F70" s="23"/>
-      <c r="G70" s="23"/>
-      <c r="H70" s="24"/>
+      <c r="A70" s="11"/>
+      <c r="B70" s="12"/>
+      <c r="C70" s="12"/>
+      <c r="D70" s="12"/>
+      <c r="E70" s="12"/>
+      <c r="F70" s="12"/>
+      <c r="G70" s="12"/>
+      <c r="H70" s="13"/>
       <c r="I70" s="1"/>
       <c r="J70" s="1"/>
       <c r="K70" s="1"/>
@@ -2950,16 +2866,14 @@
       <c r="Z70" s="1"/>
     </row>
     <row r="71" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="38" t="s">
-        <v>59</v>
-      </c>
-      <c r="B71" s="23"/>
-      <c r="C71" s="23"/>
-      <c r="D71" s="23"/>
-      <c r="E71" s="23"/>
-      <c r="F71" s="23"/>
-      <c r="G71" s="23"/>
-      <c r="H71" s="24"/>
+      <c r="A71" s="11"/>
+      <c r="B71" s="12"/>
+      <c r="C71" s="12"/>
+      <c r="D71" s="12"/>
+      <c r="E71" s="12"/>
+      <c r="F71" s="12"/>
+      <c r="G71" s="12"/>
+      <c r="H71" s="13"/>
       <c r="I71" s="1"/>
       <c r="J71" s="1"/>
       <c r="K71" s="1"/>
@@ -2980,16 +2894,14 @@
       <c r="Z71" s="1"/>
     </row>
     <row r="72" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="38" t="s">
-        <v>60</v>
-      </c>
-      <c r="B72" s="23"/>
-      <c r="C72" s="23"/>
-      <c r="D72" s="23"/>
-      <c r="E72" s="23"/>
-      <c r="F72" s="23"/>
-      <c r="G72" s="23"/>
-      <c r="H72" s="24"/>
+      <c r="A72" s="11"/>
+      <c r="B72" s="12"/>
+      <c r="C72" s="12"/>
+      <c r="D72" s="12"/>
+      <c r="E72" s="12"/>
+      <c r="F72" s="12"/>
+      <c r="G72" s="12"/>
+      <c r="H72" s="13"/>
       <c r="I72" s="1"/>
       <c r="J72" s="1"/>
       <c r="K72" s="1"/>
@@ -3010,46 +2922,42 @@
       <c r="Z72" s="1"/>
     </row>
     <row r="73" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="38" t="s">
-        <v>61</v>
-      </c>
-      <c r="B73" s="23"/>
-      <c r="C73" s="23"/>
-      <c r="D73" s="23"/>
-      <c r="E73" s="23"/>
-      <c r="F73" s="23"/>
-      <c r="G73" s="23"/>
-      <c r="H73" s="24"/>
-      <c r="I73" s="1"/>
-      <c r="J73" s="1"/>
-      <c r="K73" s="1"/>
-      <c r="L73" s="1"/>
-      <c r="M73" s="1"/>
-      <c r="N73" s="1"/>
-      <c r="O73" s="1"/>
-      <c r="P73" s="1"/>
-      <c r="Q73" s="1"/>
-      <c r="R73" s="1"/>
-      <c r="S73" s="1"/>
-      <c r="T73" s="1"/>
-      <c r="U73" s="1"/>
-      <c r="V73" s="1"/>
-      <c r="W73" s="1"/>
-      <c r="X73" s="1"/>
-      <c r="Y73" s="1"/>
-      <c r="Z73" s="1"/>
+      <c r="A73" s="14"/>
+      <c r="B73" s="12"/>
+      <c r="C73" s="12"/>
+      <c r="D73" s="12"/>
+      <c r="E73" s="12"/>
+      <c r="F73" s="12"/>
+      <c r="G73" s="12"/>
+      <c r="H73" s="13"/>
+      <c r="I73" s="4"/>
+      <c r="J73" s="4"/>
+      <c r="K73" s="4"/>
+      <c r="L73" s="4"/>
+      <c r="M73" s="4"/>
+      <c r="N73" s="4"/>
+      <c r="O73" s="4"/>
+      <c r="P73" s="4"/>
+      <c r="Q73" s="4"/>
+      <c r="R73" s="4"/>
+      <c r="S73" s="4"/>
+      <c r="T73" s="4"/>
+      <c r="U73" s="4"/>
+      <c r="V73" s="4"/>
+      <c r="W73" s="4"/>
+      <c r="X73" s="4"/>
+      <c r="Y73" s="4"/>
+      <c r="Z73" s="4"/>
     </row>
     <row r="74" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="37" t="s">
-        <v>62</v>
-      </c>
-      <c r="B74" s="23"/>
-      <c r="C74" s="23"/>
-      <c r="D74" s="23"/>
-      <c r="E74" s="23"/>
-      <c r="F74" s="23"/>
-      <c r="G74" s="23"/>
-      <c r="H74" s="24"/>
+      <c r="A74" s="1"/>
+      <c r="B74" s="1"/>
+      <c r="C74" s="1"/>
+      <c r="D74" s="1"/>
+      <c r="E74" s="1"/>
+      <c r="F74" s="1"/>
+      <c r="G74" s="1"/>
+      <c r="H74" s="1"/>
       <c r="I74" s="1"/>
       <c r="J74" s="1"/>
       <c r="K74" s="1"/>
@@ -3070,16 +2978,14 @@
       <c r="Z74" s="1"/>
     </row>
     <row r="75" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="38" t="s">
-        <v>63</v>
-      </c>
-      <c r="B75" s="23"/>
-      <c r="C75" s="23"/>
-      <c r="D75" s="23"/>
-      <c r="E75" s="23"/>
-      <c r="F75" s="23"/>
-      <c r="G75" s="23"/>
-      <c r="H75" s="24"/>
+      <c r="A75" s="1"/>
+      <c r="B75" s="1"/>
+      <c r="C75" s="1"/>
+      <c r="D75" s="1"/>
+      <c r="E75" s="1"/>
+      <c r="F75" s="1"/>
+      <c r="G75" s="1"/>
+      <c r="H75" s="1"/>
       <c r="I75" s="1"/>
       <c r="J75" s="1"/>
       <c r="K75" s="1"/>
@@ -3100,16 +3006,14 @@
       <c r="Z75" s="1"/>
     </row>
     <row r="76" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="38" t="s">
-        <v>60</v>
-      </c>
-      <c r="B76" s="23"/>
-      <c r="C76" s="23"/>
-      <c r="D76" s="23"/>
-      <c r="E76" s="23"/>
-      <c r="F76" s="23"/>
-      <c r="G76" s="23"/>
-      <c r="H76" s="24"/>
+      <c r="A76" s="1"/>
+      <c r="B76" s="1"/>
+      <c r="C76" s="1"/>
+      <c r="D76" s="1"/>
+      <c r="E76" s="1"/>
+      <c r="F76" s="1"/>
+      <c r="G76" s="1"/>
+      <c r="H76" s="1"/>
       <c r="I76" s="1"/>
       <c r="J76" s="1"/>
       <c r="K76" s="1"/>
@@ -3130,16 +3034,14 @@
       <c r="Z76" s="1"/>
     </row>
     <row r="77" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="38" t="s">
-        <v>64</v>
-      </c>
-      <c r="B77" s="23"/>
-      <c r="C77" s="23"/>
-      <c r="D77" s="23"/>
-      <c r="E77" s="23"/>
-      <c r="F77" s="23"/>
-      <c r="G77" s="23"/>
-      <c r="H77" s="24"/>
+      <c r="A77" s="1"/>
+      <c r="B77" s="1"/>
+      <c r="C77" s="1"/>
+      <c r="D77" s="1"/>
+      <c r="E77" s="1"/>
+      <c r="F77" s="1"/>
+      <c r="G77" s="1"/>
+      <c r="H77" s="1"/>
       <c r="I77" s="1"/>
       <c r="J77" s="1"/>
       <c r="K77" s="1"/>
@@ -3160,34 +3062,32 @@
       <c r="Z77" s="1"/>
     </row>
     <row r="78" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="39" t="s">
-        <v>65</v>
-      </c>
-      <c r="B78" s="23"/>
-      <c r="C78" s="23"/>
-      <c r="D78" s="23"/>
-      <c r="E78" s="23"/>
-      <c r="F78" s="23"/>
-      <c r="G78" s="23"/>
-      <c r="H78" s="24"/>
-      <c r="I78" s="6"/>
-      <c r="J78" s="6"/>
-      <c r="K78" s="6"/>
-      <c r="L78" s="6"/>
-      <c r="M78" s="6"/>
-      <c r="N78" s="6"/>
-      <c r="O78" s="6"/>
-      <c r="P78" s="6"/>
-      <c r="Q78" s="6"/>
-      <c r="R78" s="6"/>
-      <c r="S78" s="6"/>
-      <c r="T78" s="6"/>
-      <c r="U78" s="6"/>
-      <c r="V78" s="6"/>
-      <c r="W78" s="6"/>
-      <c r="X78" s="6"/>
-      <c r="Y78" s="6"/>
-      <c r="Z78" s="6"/>
+      <c r="A78" s="1"/>
+      <c r="B78" s="1"/>
+      <c r="C78" s="1"/>
+      <c r="D78" s="1"/>
+      <c r="E78" s="1"/>
+      <c r="F78" s="1"/>
+      <c r="G78" s="1"/>
+      <c r="H78" s="1"/>
+      <c r="I78" s="1"/>
+      <c r="J78" s="1"/>
+      <c r="K78" s="1"/>
+      <c r="L78" s="1"/>
+      <c r="M78" s="1"/>
+      <c r="N78" s="1"/>
+      <c r="O78" s="1"/>
+      <c r="P78" s="1"/>
+      <c r="Q78" s="1"/>
+      <c r="R78" s="1"/>
+      <c r="S78" s="1"/>
+      <c r="T78" s="1"/>
+      <c r="U78" s="1"/>
+      <c r="V78" s="1"/>
+      <c r="W78" s="1"/>
+      <c r="X78" s="1"/>
+      <c r="Y78" s="1"/>
+      <c r="Z78" s="1"/>
     </row>
     <row r="79" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1"/>
@@ -7277,212 +7177,69 @@
       <c r="Y224" s="1"/>
       <c r="Z224" s="1"/>
     </row>
-    <row r="225" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A225" s="1"/>
-      <c r="B225" s="1"/>
-      <c r="C225" s="1"/>
-      <c r="D225" s="1"/>
-      <c r="E225" s="1"/>
-      <c r="F225" s="1"/>
-      <c r="G225" s="1"/>
-      <c r="H225" s="1"/>
-      <c r="I225" s="1"/>
-      <c r="J225" s="1"/>
-      <c r="K225" s="1"/>
-      <c r="L225" s="1"/>
-      <c r="M225" s="1"/>
-      <c r="N225" s="1"/>
-      <c r="O225" s="1"/>
-      <c r="P225" s="1"/>
-      <c r="Q225" s="1"/>
-      <c r="R225" s="1"/>
-      <c r="S225" s="1"/>
-      <c r="T225" s="1"/>
-      <c r="U225" s="1"/>
-      <c r="V225" s="1"/>
-      <c r="W225" s="1"/>
-      <c r="X225" s="1"/>
-      <c r="Y225" s="1"/>
-      <c r="Z225" s="1"/>
-    </row>
-    <row r="226" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A226" s="1"/>
-      <c r="B226" s="1"/>
-      <c r="C226" s="1"/>
-      <c r="D226" s="1"/>
-      <c r="E226" s="1"/>
-      <c r="F226" s="1"/>
-      <c r="G226" s="1"/>
-      <c r="H226" s="1"/>
-      <c r="I226" s="1"/>
-      <c r="J226" s="1"/>
-      <c r="K226" s="1"/>
-      <c r="L226" s="1"/>
-      <c r="M226" s="1"/>
-      <c r="N226" s="1"/>
-      <c r="O226" s="1"/>
-      <c r="P226" s="1"/>
-      <c r="Q226" s="1"/>
-      <c r="R226" s="1"/>
-      <c r="S226" s="1"/>
-      <c r="T226" s="1"/>
-      <c r="U226" s="1"/>
-      <c r="V226" s="1"/>
-      <c r="W226" s="1"/>
-      <c r="X226" s="1"/>
-      <c r="Y226" s="1"/>
-      <c r="Z226" s="1"/>
-    </row>
-    <row r="227" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A227" s="1"/>
-      <c r="B227" s="1"/>
-      <c r="C227" s="1"/>
-      <c r="D227" s="1"/>
-      <c r="E227" s="1"/>
-      <c r="F227" s="1"/>
-      <c r="G227" s="1"/>
-      <c r="H227" s="1"/>
-      <c r="I227" s="1"/>
-      <c r="J227" s="1"/>
-      <c r="K227" s="1"/>
-      <c r="L227" s="1"/>
-      <c r="M227" s="1"/>
-      <c r="N227" s="1"/>
-      <c r="O227" s="1"/>
-      <c r="P227" s="1"/>
-      <c r="Q227" s="1"/>
-      <c r="R227" s="1"/>
-      <c r="S227" s="1"/>
-      <c r="T227" s="1"/>
-      <c r="U227" s="1"/>
-      <c r="V227" s="1"/>
-      <c r="W227" s="1"/>
-      <c r="X227" s="1"/>
-      <c r="Y227" s="1"/>
-      <c r="Z227" s="1"/>
-    </row>
-    <row r="228" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A228" s="1"/>
-      <c r="B228" s="1"/>
-      <c r="C228" s="1"/>
-      <c r="D228" s="1"/>
-      <c r="E228" s="1"/>
-      <c r="F228" s="1"/>
-      <c r="G228" s="1"/>
-      <c r="H228" s="1"/>
-      <c r="I228" s="1"/>
-      <c r="J228" s="1"/>
-      <c r="K228" s="1"/>
-      <c r="L228" s="1"/>
-      <c r="M228" s="1"/>
-      <c r="N228" s="1"/>
-      <c r="O228" s="1"/>
-      <c r="P228" s="1"/>
-      <c r="Q228" s="1"/>
-      <c r="R228" s="1"/>
-      <c r="S228" s="1"/>
-      <c r="T228" s="1"/>
-      <c r="U228" s="1"/>
-      <c r="V228" s="1"/>
-      <c r="W228" s="1"/>
-      <c r="X228" s="1"/>
-      <c r="Y228" s="1"/>
-      <c r="Z228" s="1"/>
-    </row>
-    <row r="229" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A229" s="1"/>
-      <c r="B229" s="1"/>
-      <c r="C229" s="1"/>
-      <c r="D229" s="1"/>
-      <c r="E229" s="1"/>
-      <c r="F229" s="1"/>
-      <c r="G229" s="1"/>
-      <c r="H229" s="1"/>
-      <c r="I229" s="1"/>
-      <c r="J229" s="1"/>
-      <c r="K229" s="1"/>
-      <c r="L229" s="1"/>
-      <c r="M229" s="1"/>
-      <c r="N229" s="1"/>
-      <c r="O229" s="1"/>
-      <c r="P229" s="1"/>
-      <c r="Q229" s="1"/>
-      <c r="R229" s="1"/>
-      <c r="S229" s="1"/>
-      <c r="T229" s="1"/>
-      <c r="U229" s="1"/>
-      <c r="V229" s="1"/>
-      <c r="W229" s="1"/>
-      <c r="X229" s="1"/>
-      <c r="Y229" s="1"/>
-      <c r="Z229" s="1"/>
-    </row>
   </sheetData>
-  <mergeCells count="60">
-    <mergeCell ref="A76:H76"/>
-    <mergeCell ref="A77:H77"/>
-    <mergeCell ref="A78:H78"/>
-    <mergeCell ref="A71:H71"/>
-    <mergeCell ref="A72:H72"/>
-    <mergeCell ref="A73:H73"/>
-    <mergeCell ref="A74:H74"/>
-    <mergeCell ref="A75:H75"/>
-    <mergeCell ref="B66:G66"/>
-    <mergeCell ref="B67:G67"/>
-    <mergeCell ref="B68:G68"/>
-    <mergeCell ref="B69:G69"/>
-    <mergeCell ref="A70:H70"/>
-    <mergeCell ref="B61:G61"/>
-    <mergeCell ref="B62:G62"/>
-    <mergeCell ref="B63:G63"/>
-    <mergeCell ref="B64:G64"/>
-    <mergeCell ref="B65:G65"/>
-    <mergeCell ref="A56:H56"/>
+  <mergeCells count="58">
+    <mergeCell ref="A1:H2"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="E35:F35"/>
+    <mergeCell ref="G35:H35"/>
+    <mergeCell ref="A37:C37"/>
+    <mergeCell ref="E37:H37"/>
+    <mergeCell ref="F38:H38"/>
+    <mergeCell ref="F39:H39"/>
+    <mergeCell ref="F40:H40"/>
+    <mergeCell ref="F41:H41"/>
+    <mergeCell ref="F42:H42"/>
+    <mergeCell ref="F43:H43"/>
+    <mergeCell ref="F44:H44"/>
+    <mergeCell ref="F45:H45"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="F46:H46"/>
+    <mergeCell ref="A48:H48"/>
+    <mergeCell ref="B49:G49"/>
+    <mergeCell ref="B50:G50"/>
+    <mergeCell ref="B51:G51"/>
+    <mergeCell ref="B52:G52"/>
+    <mergeCell ref="B53:G53"/>
+    <mergeCell ref="B54:G54"/>
+    <mergeCell ref="B55:G55"/>
+    <mergeCell ref="B56:G56"/>
     <mergeCell ref="B57:G57"/>
     <mergeCell ref="B58:G58"/>
     <mergeCell ref="B59:G59"/>
     <mergeCell ref="B60:G60"/>
-    <mergeCell ref="F51:H51"/>
-    <mergeCell ref="F52:H52"/>
-    <mergeCell ref="F53:H53"/>
-    <mergeCell ref="B54:C54"/>
-    <mergeCell ref="F54:H54"/>
-    <mergeCell ref="F46:H46"/>
-    <mergeCell ref="F47:H47"/>
-    <mergeCell ref="F48:H48"/>
-    <mergeCell ref="F49:H49"/>
-    <mergeCell ref="F50:H50"/>
-    <mergeCell ref="A43:B43"/>
-    <mergeCell ref="C43:D43"/>
-    <mergeCell ref="E43:F43"/>
-    <mergeCell ref="G43:H43"/>
-    <mergeCell ref="A45:C45"/>
-    <mergeCell ref="E45:H45"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="E30:F30"/>
-    <mergeCell ref="G30:H30"/>
-    <mergeCell ref="A17:H17"/>
-    <mergeCell ref="A12:H12"/>
-    <mergeCell ref="A13:B16"/>
-    <mergeCell ref="C13:H13"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="A1:H2"/>
-    <mergeCell ref="A3:B11"/>
-    <mergeCell ref="D3:H3"/>
-    <mergeCell ref="D4:H4"/>
-    <mergeCell ref="D5:H5"/>
-    <mergeCell ref="D6:H6"/>
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D9:H9"/>
-    <mergeCell ref="D10:H10"/>
-    <mergeCell ref="D11:H11"/>
+    <mergeCell ref="B61:G61"/>
+    <mergeCell ref="A62:H62"/>
+    <mergeCell ref="A70:H70"/>
+    <mergeCell ref="A72:H72"/>
+    <mergeCell ref="A73:H73"/>
+    <mergeCell ref="A63:H63"/>
+    <mergeCell ref="A66:H66"/>
+    <mergeCell ref="A67:H67"/>
+    <mergeCell ref="A68:H68"/>
+    <mergeCell ref="A69:H69"/>
+    <mergeCell ref="A64:H64"/>
+    <mergeCell ref="A65:H65"/>
+    <mergeCell ref="A71:H71"/>
   </mergeCells>
   <printOptions horizontalCentered="1" gridLines="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="14" pageOrder="overThenDown" orientation="portrait" cellComments="atEnd"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>